<commit_message>
corrections forestgeo current names in plantnet list, alternate names problems and garwood modifications for hybrids
</commit_message>
<xml_diff>
--- a/splists_out/ViewTaxonomy_dec4_25_SYNONYMS.xlsx
+++ b/splists_out/ViewTaxonomy_dec4_25_SYNONYMS.xlsx
@@ -398,7 +398,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>396</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -436,7 +436,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>1025</v>
+        <v>12</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>1026</v>
+        <v>13</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -512,7 +512,7 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>535</v>
+        <v>14</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -550,7 +550,7 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>536</v>
+        <v>15</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>323</v>
+        <v>18</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>1027</v>
+        <v>23</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
     </row>
     <row r="9">
       <c r="A9">
-        <v>1029</v>
+        <v>29</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -702,7 +702,7 @@
     </row>
     <row r="10">
       <c r="A10">
-        <v>1030</v>
+        <v>30</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
     </row>
     <row r="11">
       <c r="A11">
-        <v>537</v>
+        <v>47</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
     </row>
     <row r="14">
       <c r="A14">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
     </row>
     <row r="15">
       <c r="A15">
-        <v>638</v>
+        <v>64</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
     </row>
     <row r="16">
       <c r="A16">
-        <v>1035</v>
+        <v>70</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
     </row>
     <row r="17">
       <c r="A17">
-        <v>100</v>
+        <v>71</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1006,7 +1006,7 @@
     </row>
     <row r="18">
       <c r="A18">
-        <v>863</v>
+        <v>74</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="19">
       <c r="A19">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="20">
       <c r="A20">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
     </row>
     <row r="21">
       <c r="A21">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="22">
       <c r="A22">
-        <v>542</v>
+        <v>108</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
     </row>
     <row r="23">
       <c r="A23">
-        <v>543</v>
+        <v>109</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
     </row>
     <row r="24">
       <c r="A24">
-        <v>1322</v>
+        <v>118</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="25">
       <c r="A25">
-        <v>1401</v>
+        <v>121</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="26">
       <c r="A26">
-        <v>1402</v>
+        <v>122</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     </row>
     <row r="27">
       <c r="A27">
-        <v>792</v>
+        <v>127</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
     </row>
     <row r="28">
       <c r="A28">
-        <v>626</v>
+        <v>132</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="29">
       <c r="A29">
-        <v>631</v>
+        <v>139</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1462,7 +1462,7 @@
     </row>
     <row r="30">
       <c r="A30">
-        <v>400</v>
+        <v>143</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="31">
       <c r="A31">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1538,7 +1538,7 @@
     </row>
     <row r="32">
       <c r="A32">
-        <v>1177</v>
+        <v>159</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
     </row>
     <row r="33">
       <c r="A33">
-        <v>1177</v>
+        <v>159</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
     </row>
     <row r="34">
       <c r="A34">
-        <v>1177</v>
+        <v>159</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1652,7 +1652,7 @@
     </row>
     <row r="35">
       <c r="A35">
-        <v>1179</v>
+        <v>161</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
     </row>
     <row r="36">
       <c r="A36">
-        <v>1183</v>
+        <v>165</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
     </row>
     <row r="37">
       <c r="A37">
-        <v>1020</v>
+        <v>174</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="38">
       <c r="A38">
-        <v>640</v>
+        <v>178</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
     </row>
     <row r="39">
       <c r="A39">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1842,7 +1842,7 @@
     </row>
     <row r="40">
       <c r="A40">
-        <v>945</v>
+        <v>191</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1880,7 +1880,7 @@
     </row>
     <row r="41">
       <c r="A41">
-        <v>1304</v>
+        <v>194</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
     </row>
     <row r="42">
       <c r="A42">
-        <v>122</v>
+        <v>196</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
     </row>
     <row r="43">
       <c r="A43">
-        <v>887</v>
+        <v>197</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="44">
       <c r="A44">
-        <v>1231</v>
+        <v>204</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="45">
       <c r="A45">
-        <v>239</v>
+        <v>208</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
     </row>
     <row r="46">
       <c r="A46">
-        <v>1232</v>
+        <v>209</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
     </row>
     <row r="47">
       <c r="A47">
-        <v>1232</v>
+        <v>209</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
     </row>
     <row r="48">
       <c r="A48">
-        <v>1158</v>
+        <v>219</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -2184,7 +2184,7 @@
     </row>
     <row r="49">
       <c r="A49">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
     </row>
     <row r="50">
       <c r="A50">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
     </row>
     <row r="51">
       <c r="A51">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
     </row>
     <row r="52">
       <c r="A52">
-        <v>403</v>
+        <v>252</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -2336,7 +2336,7 @@
     </row>
     <row r="53">
       <c r="A53">
-        <v>843</v>
+        <v>257</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -2374,7 +2374,7 @@
     </row>
     <row r="54">
       <c r="A54">
-        <v>844</v>
+        <v>258</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -2412,7 +2412,7 @@
     </row>
     <row r="55">
       <c r="A55">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
     </row>
     <row r="56">
       <c r="A56">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -2488,7 +2488,7 @@
     </row>
     <row r="57">
       <c r="A57">
-        <v>1044</v>
+        <v>280</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
     </row>
     <row r="58">
       <c r="A58">
-        <v>1050</v>
+        <v>290</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="59">
       <c r="A59">
-        <v>40</v>
+        <v>293</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -2602,7 +2602,7 @@
     </row>
     <row r="60">
       <c r="A60">
-        <v>332</v>
+        <v>300</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="61">
       <c r="A61">
-        <v>546</v>
+        <v>308</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
     </row>
     <row r="62">
       <c r="A62">
-        <v>1213</v>
+        <v>311</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
     </row>
     <row r="63">
       <c r="A63">
-        <v>1216</v>
+        <v>314</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -2754,7 +2754,7 @@
     </row>
     <row r="64">
       <c r="A64">
-        <v>294</v>
+        <v>321</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="65">
       <c r="A65">
-        <v>547</v>
+        <v>328</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2830,7 +2830,7 @@
     </row>
     <row r="66">
       <c r="A66">
-        <v>548</v>
+        <v>329</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2868,7 +2868,7 @@
     </row>
     <row r="67">
       <c r="A67">
-        <v>549</v>
+        <v>330</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2906,7 +2906,7 @@
     </row>
     <row r="68">
       <c r="A68">
-        <v>550</v>
+        <v>331</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2944,7 +2944,7 @@
     </row>
     <row r="69">
       <c r="A69">
-        <v>101</v>
+        <v>335</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2982,7 +2982,7 @@
     </row>
     <row r="70">
       <c r="A70">
-        <v>105</v>
+        <v>343</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
     </row>
     <row r="71">
       <c r="A71">
-        <v>471</v>
+        <v>348</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="72">
       <c r="A72">
-        <v>472</v>
+        <v>356</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -3096,7 +3096,7 @@
     </row>
     <row r="73">
       <c r="A73">
-        <v>318</v>
+        <v>379</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -3134,7 +3134,7 @@
     </row>
     <row r="74">
       <c r="A74">
-        <v>600</v>
+        <v>383</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
     </row>
     <row r="75">
       <c r="A75">
-        <v>601</v>
+        <v>384</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -3210,7 +3210,7 @@
     </row>
     <row r="76">
       <c r="A76">
-        <v>604</v>
+        <v>387</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     </row>
     <row r="77">
       <c r="A77">
-        <v>891</v>
+        <v>396</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -3286,7 +3286,7 @@
     </row>
     <row r="78">
       <c r="A78">
-        <v>893</v>
+        <v>398</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
@@ -3324,7 +3324,7 @@
     </row>
     <row r="79">
       <c r="A79">
-        <v>897</v>
+        <v>402</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
     </row>
     <row r="80">
       <c r="A80">
-        <v>338</v>
+        <v>419</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
     </row>
     <row r="81">
       <c r="A81">
-        <v>360</v>
+        <v>421</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -3438,7 +3438,7 @@
     </row>
     <row r="82">
       <c r="A82">
-        <v>1054</v>
+        <v>422</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -3476,7 +3476,7 @@
     </row>
     <row r="83">
       <c r="A83">
-        <v>1059</v>
+        <v>427</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -3514,7 +3514,7 @@
     </row>
     <row r="84">
       <c r="A84">
-        <v>797</v>
+        <v>434</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
     </row>
     <row r="85">
       <c r="A85">
-        <v>804</v>
+        <v>441</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -3590,7 +3590,7 @@
     </row>
     <row r="86">
       <c r="A86">
-        <v>805</v>
+        <v>442</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -3628,7 +3628,7 @@
     </row>
     <row r="87">
       <c r="A87">
-        <v>808</v>
+        <v>445</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -3666,7 +3666,7 @@
     </row>
     <row r="88">
       <c r="A88">
-        <v>822</v>
+        <v>459</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
     </row>
     <row r="89">
       <c r="A89">
-        <v>246</v>
+        <v>465</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -3742,7 +3742,7 @@
     </row>
     <row r="90">
       <c r="A90">
-        <v>246</v>
+        <v>465</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -3780,7 +3780,7 @@
     </row>
     <row r="91">
       <c r="A91">
-        <v>247</v>
+        <v>466</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -3818,7 +3818,7 @@
     </row>
     <row r="92">
       <c r="A92">
-        <v>247</v>
+        <v>466</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -3856,7 +3856,7 @@
     </row>
     <row r="93">
       <c r="A93">
-        <v>339</v>
+        <v>474</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -3894,7 +3894,7 @@
     </row>
     <row r="94">
       <c r="A94">
-        <v>1320</v>
+        <v>482</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
     </row>
     <row r="95">
       <c r="A95">
-        <v>935</v>
+        <v>490</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -3970,7 +3970,7 @@
     </row>
     <row r="96">
       <c r="A96">
-        <v>758</v>
+        <v>492</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="97">
       <c r="A97">
-        <v>759</v>
+        <v>493</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
     </row>
     <row r="98">
       <c r="A98">
-        <v>762</v>
+        <v>496</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -4084,7 +4084,7 @@
     </row>
     <row r="99">
       <c r="A99">
-        <v>764</v>
+        <v>498</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -4122,7 +4122,7 @@
     </row>
     <row r="100">
       <c r="A100">
-        <v>52</v>
+        <v>509</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -4160,7 +4160,7 @@
     </row>
     <row r="101">
       <c r="A101">
-        <v>55</v>
+        <v>512</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     </row>
     <row r="102">
       <c r="A102">
-        <v>59</v>
+        <v>516</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -4236,7 +4236,7 @@
     </row>
     <row r="103">
       <c r="A103">
-        <v>1070</v>
+        <v>518</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -4274,7 +4274,7 @@
     </row>
     <row r="104">
       <c r="A104">
-        <v>610</v>
+        <v>521</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -4312,7 +4312,7 @@
     </row>
     <row r="105">
       <c r="A105">
-        <v>645</v>
+        <v>530</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -4350,7 +4350,7 @@
     </row>
     <row r="106">
       <c r="A106">
-        <v>152</v>
+        <v>532</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -4388,7 +4388,7 @@
     </row>
     <row r="107">
       <c r="A107">
-        <v>153</v>
+        <v>533</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -4426,7 +4426,7 @@
     </row>
     <row r="108">
       <c r="A108">
-        <v>154</v>
+        <v>534</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -4464,7 +4464,7 @@
     </row>
     <row r="109">
       <c r="A109">
-        <v>691</v>
+        <v>544</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -4502,7 +4502,7 @@
     </row>
     <row r="110">
       <c r="A110">
-        <v>693</v>
+        <v>546</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -4540,7 +4540,7 @@
     </row>
     <row r="111">
       <c r="A111">
-        <v>694</v>
+        <v>547</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -4578,7 +4578,7 @@
     </row>
     <row r="112">
       <c r="A112">
-        <v>651</v>
+        <v>553</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -4616,7 +4616,7 @@
     </row>
     <row r="113">
       <c r="A113">
-        <v>341</v>
+        <v>554</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -4654,7 +4654,7 @@
     </row>
     <row r="114">
       <c r="A114">
-        <v>217</v>
+        <v>563</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -4692,7 +4692,7 @@
     </row>
     <row r="115">
       <c r="A115">
-        <v>1289</v>
+        <v>567</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -4730,7 +4730,7 @@
     </row>
     <row r="116">
       <c r="A116">
-        <v>1162</v>
+        <v>568</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
     </row>
     <row r="117">
       <c r="A117">
-        <v>878</v>
+        <v>573</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -4806,7 +4806,7 @@
     </row>
     <row r="118">
       <c r="A118">
-        <v>406</v>
+        <v>578</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -4844,7 +4844,7 @@
     </row>
     <row r="119">
       <c r="A119">
-        <v>406</v>
+        <v>578</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
     </row>
     <row r="120">
       <c r="A120">
-        <v>406</v>
+        <v>578</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -4920,7 +4920,7 @@
     </row>
     <row r="121">
       <c r="A121">
-        <v>406</v>
+        <v>578</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
     </row>
     <row r="122">
       <c r="A122">
-        <v>413</v>
+        <v>585</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -4996,7 +4996,7 @@
     </row>
     <row r="123">
       <c r="A123">
-        <v>419</v>
+        <v>591</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -5034,7 +5034,7 @@
     </row>
     <row r="124">
       <c r="A124">
-        <v>420</v>
+        <v>592</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -5072,7 +5072,7 @@
     </row>
     <row r="125">
       <c r="A125">
-        <v>420</v>
+        <v>592</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -5110,7 +5110,7 @@
     </row>
     <row r="126">
       <c r="A126">
-        <v>425</v>
+        <v>597</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     </row>
     <row r="127">
       <c r="A127">
-        <v>426</v>
+        <v>598</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -5186,7 +5186,7 @@
     </row>
     <row r="128">
       <c r="A128">
-        <v>447</v>
+        <v>619</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -5224,7 +5224,7 @@
     </row>
     <row r="129">
       <c r="A129">
-        <v>448</v>
+        <v>620</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -5262,7 +5262,7 @@
     </row>
     <row r="130">
       <c r="A130">
-        <v>448</v>
+        <v>620</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -5300,7 +5300,7 @@
     </row>
     <row r="131">
       <c r="A131">
-        <v>1079</v>
+        <v>629</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -5338,7 +5338,7 @@
     </row>
     <row r="132">
       <c r="A132">
-        <v>198</v>
+        <v>632</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -5376,7 +5376,7 @@
     </row>
     <row r="133">
       <c r="A133">
-        <v>525</v>
+        <v>642</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
     </row>
     <row r="134">
       <c r="A134">
-        <v>83</v>
+        <v>652</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -5452,7 +5452,7 @@
     </row>
     <row r="135">
       <c r="A135">
-        <v>1405</v>
+        <v>657</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -5490,7 +5490,7 @@
     </row>
     <row r="136">
       <c r="A136">
-        <v>1406</v>
+        <v>658</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -5528,7 +5528,7 @@
     </row>
     <row r="137">
       <c r="A137">
-        <v>1408</v>
+        <v>660</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -5566,7 +5566,7 @@
     </row>
     <row r="138">
       <c r="A138">
-        <v>219</v>
+        <v>661</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -5604,7 +5604,7 @@
     </row>
     <row r="139">
       <c r="A139">
-        <v>364</v>
+        <v>662</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
     </row>
     <row r="140">
       <c r="A140">
-        <v>180</v>
+        <v>663</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -5680,7 +5680,7 @@
     </row>
     <row r="141">
       <c r="A141">
-        <v>365</v>
+        <v>664</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -5718,7 +5718,7 @@
     </row>
     <row r="142">
       <c r="A142">
-        <v>492</v>
+        <v>680</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -5756,7 +5756,7 @@
     </row>
     <row r="143">
       <c r="A143">
-        <v>1082</v>
+        <v>692</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -5794,7 +5794,7 @@
     </row>
     <row r="144">
       <c r="A144">
-        <v>824</v>
+        <v>693</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -5832,7 +5832,7 @@
     </row>
     <row r="145">
       <c r="A145">
-        <v>1083</v>
+        <v>695</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -5870,7 +5870,7 @@
     </row>
     <row r="146">
       <c r="A146">
-        <v>622</v>
+        <v>699</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
     </row>
     <row r="147">
       <c r="A147">
-        <v>623</v>
+        <v>700</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
@@ -5946,7 +5946,7 @@
     </row>
     <row r="148">
       <c r="A148">
-        <v>86</v>
+        <v>703</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
@@ -5984,7 +5984,7 @@
     </row>
     <row r="149">
       <c r="A149">
-        <v>825</v>
+        <v>715</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -6022,7 +6022,7 @@
     </row>
     <row r="150">
       <c r="A150">
-        <v>959</v>
+        <v>717</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -6060,7 +6060,7 @@
     </row>
     <row r="151">
       <c r="A151">
-        <v>253</v>
+        <v>720</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     </row>
     <row r="152">
       <c r="A152">
-        <v>254</v>
+        <v>721</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -6136,7 +6136,7 @@
     </row>
     <row r="153">
       <c r="A153">
-        <v>1223</v>
+        <v>725</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
     </row>
     <row r="154">
       <c r="A154">
-        <v>656</v>
+        <v>730</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -6212,7 +6212,7 @@
     </row>
     <row r="155">
       <c r="A155">
-        <v>202</v>
+        <v>736</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -6250,7 +6250,7 @@
     </row>
     <row r="156">
       <c r="A156">
-        <v>1174</v>
+        <v>745</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -6288,7 +6288,7 @@
     </row>
     <row r="157">
       <c r="A157">
-        <v>557</v>
+        <v>746</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -6326,7 +6326,7 @@
     </row>
     <row r="158">
       <c r="A158">
-        <v>558</v>
+        <v>747</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -6364,7 +6364,7 @@
     </row>
     <row r="159">
       <c r="A159">
-        <v>696</v>
+        <v>748</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -6402,7 +6402,7 @@
     </row>
     <row r="160">
       <c r="A160">
-        <v>698</v>
+        <v>750</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
     </row>
     <row r="161">
       <c r="A161">
-        <v>703</v>
+        <v>755</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -6478,7 +6478,7 @@
     </row>
     <row r="162">
       <c r="A162">
-        <v>704</v>
+        <v>756</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -6516,7 +6516,7 @@
     </row>
     <row r="163">
       <c r="A163">
-        <v>705</v>
+        <v>757</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -6554,7 +6554,7 @@
     </row>
     <row r="164">
       <c r="A164">
-        <v>706</v>
+        <v>758</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -6592,7 +6592,7 @@
     </row>
     <row r="165">
       <c r="A165">
-        <v>707</v>
+        <v>759</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -6630,7 +6630,7 @@
     </row>
     <row r="166">
       <c r="A166">
-        <v>708</v>
+        <v>760</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -6668,7 +6668,7 @@
     </row>
     <row r="167">
       <c r="A167">
-        <v>709</v>
+        <v>761</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -6706,7 +6706,7 @@
     </row>
     <row r="168">
       <c r="A168">
-        <v>710</v>
+        <v>762</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -6744,7 +6744,7 @@
     </row>
     <row r="169">
       <c r="A169">
-        <v>711</v>
+        <v>763</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -6782,7 +6782,7 @@
     </row>
     <row r="170">
       <c r="A170">
-        <v>713</v>
+        <v>765</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -6820,7 +6820,7 @@
     </row>
     <row r="171">
       <c r="A171">
-        <v>714</v>
+        <v>766</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -6858,7 +6858,7 @@
     </row>
     <row r="172">
       <c r="A172">
-        <v>716</v>
+        <v>768</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
@@ -6896,7 +6896,7 @@
     </row>
     <row r="173">
       <c r="A173">
-        <v>717</v>
+        <v>769</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -6934,7 +6934,7 @@
     </row>
     <row r="174">
       <c r="A174">
-        <v>718</v>
+        <v>770</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -6972,7 +6972,7 @@
     </row>
     <row r="175">
       <c r="A175">
-        <v>726</v>
+        <v>778</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -7010,7 +7010,7 @@
     </row>
     <row r="176">
       <c r="A176">
-        <v>729</v>
+        <v>781</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     </row>
     <row r="177">
       <c r="A177">
-        <v>732</v>
+        <v>784</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -7086,7 +7086,7 @@
     </row>
     <row r="178">
       <c r="A178">
-        <v>740</v>
+        <v>792</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -7124,7 +7124,7 @@
     </row>
     <row r="179">
       <c r="A179">
-        <v>742</v>
+        <v>794</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
@@ -7162,7 +7162,7 @@
     </row>
     <row r="180">
       <c r="A180">
-        <v>743</v>
+        <v>795</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
@@ -7200,7 +7200,7 @@
     </row>
     <row r="181">
       <c r="A181">
-        <v>744</v>
+        <v>796</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -7238,7 +7238,7 @@
     </row>
     <row r="182">
       <c r="A182">
-        <v>747</v>
+        <v>799</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -7276,7 +7276,7 @@
     </row>
     <row r="183">
       <c r="A183">
-        <v>227</v>
+        <v>800</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -7314,7 +7314,7 @@
     </row>
     <row r="184">
       <c r="A184">
-        <v>786</v>
+        <v>807</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -7352,7 +7352,7 @@
     </row>
     <row r="185">
       <c r="A185">
-        <v>786</v>
+        <v>807</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -7390,7 +7390,7 @@
     </row>
     <row r="186">
       <c r="A186">
-        <v>228</v>
+        <v>808</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
     </row>
     <row r="187">
       <c r="A187">
-        <v>229</v>
+        <v>809</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -7466,7 +7466,7 @@
     </row>
     <row r="188">
       <c r="A188">
-        <v>230</v>
+        <v>810</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -7504,7 +7504,7 @@
     </row>
     <row r="189">
       <c r="A189">
-        <v>231</v>
+        <v>811</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -7542,7 +7542,7 @@
     </row>
     <row r="190">
       <c r="A190">
-        <v>1086</v>
+        <v>814</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -7580,7 +7580,7 @@
     </row>
     <row r="191">
       <c r="A191">
-        <v>187</v>
+        <v>815</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -7618,7 +7618,7 @@
     </row>
     <row r="192">
       <c r="A192">
-        <v>188</v>
+        <v>816</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -7656,7 +7656,7 @@
     </row>
     <row r="193">
       <c r="A193">
-        <v>189</v>
+        <v>817</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -7694,7 +7694,7 @@
     </row>
     <row r="194">
       <c r="A194">
-        <v>190</v>
+        <v>818</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -7732,7 +7732,7 @@
     </row>
     <row r="195">
       <c r="A195">
-        <v>191</v>
+        <v>819</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -7770,7 +7770,7 @@
     </row>
     <row r="196">
       <c r="A196">
-        <v>192</v>
+        <v>820</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -7808,7 +7808,7 @@
     </row>
     <row r="197">
       <c r="A197">
-        <v>193</v>
+        <v>821</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -7846,7 +7846,7 @@
     </row>
     <row r="198">
       <c r="A198">
-        <v>194</v>
+        <v>822</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -7884,7 +7884,7 @@
     </row>
     <row r="199">
       <c r="A199">
-        <v>195</v>
+        <v>823</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -7922,7 +7922,7 @@
     </row>
     <row r="200">
       <c r="A200">
-        <v>196</v>
+        <v>824</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -7960,7 +7960,7 @@
     </row>
     <row r="201">
       <c r="A201">
-        <v>62</v>
+        <v>827</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     </row>
     <row r="202">
       <c r="A202">
-        <v>749</v>
+        <v>830</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -8036,7 +8036,7 @@
     </row>
     <row r="203">
       <c r="A203">
-        <v>750</v>
+        <v>831</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -8074,7 +8074,7 @@
     </row>
     <row r="204">
       <c r="A204">
-        <v>914</v>
+        <v>836</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -8112,7 +8112,7 @@
     </row>
     <row r="205">
       <c r="A205">
-        <v>917</v>
+        <v>839</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -8150,7 +8150,7 @@
     </row>
     <row r="206">
       <c r="A206">
-        <v>921</v>
+        <v>843</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -8188,7 +8188,7 @@
     </row>
     <row r="207">
       <c r="A207">
-        <v>921</v>
+        <v>843</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
     </row>
     <row r="208">
       <c r="A208">
-        <v>922</v>
+        <v>844</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -8264,7 +8264,7 @@
     </row>
     <row r="209">
       <c r="A209">
-        <v>923</v>
+        <v>845</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -8302,7 +8302,7 @@
     </row>
     <row r="210">
       <c r="A210">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -8340,7 +8340,7 @@
     </row>
     <row r="211">
       <c r="A211">
-        <v>561</v>
+        <v>860</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -8378,7 +8378,7 @@
     </row>
     <row r="212">
       <c r="A212">
-        <v>562</v>
+        <v>861</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -8416,7 +8416,7 @@
     </row>
     <row r="213">
       <c r="A213">
-        <v>567</v>
+        <v>866</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -8454,7 +8454,7 @@
     </row>
     <row r="214">
       <c r="A214">
-        <v>366</v>
+        <v>877</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -8492,7 +8492,7 @@
     </row>
     <row r="215">
       <c r="A215">
-        <v>573</v>
+        <v>884</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -8530,7 +8530,7 @@
     </row>
     <row r="216">
       <c r="A216">
-        <v>574</v>
+        <v>885</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -8568,7 +8568,7 @@
     </row>
     <row r="217">
       <c r="A217">
-        <v>576</v>
+        <v>887</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -8606,7 +8606,7 @@
     </row>
     <row r="218">
       <c r="A218">
-        <v>578</v>
+        <v>889</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -8644,7 +8644,7 @@
     </row>
     <row r="219">
       <c r="A219">
-        <v>580</v>
+        <v>891</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
@@ -8682,7 +8682,7 @@
     </row>
     <row r="220">
       <c r="A220">
-        <v>591</v>
+        <v>902</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -8720,7 +8720,7 @@
     </row>
     <row r="221">
       <c r="A221">
-        <v>591</v>
+        <v>902</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
@@ -8758,7 +8758,7 @@
     </row>
     <row r="222">
       <c r="A222">
-        <v>133</v>
+        <v>903</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -8796,7 +8796,7 @@
     </row>
     <row r="223">
       <c r="A223">
-        <v>499</v>
+        <v>908</v>
       </c>
       <c r="B223" t="inlineStr">
         <is>
@@ -8834,7 +8834,7 @@
     </row>
     <row r="224">
       <c r="A224">
-        <v>665</v>
+        <v>924</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
@@ -8872,7 +8872,7 @@
     </row>
     <row r="225">
       <c r="A225">
-        <v>665</v>
+        <v>924</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
@@ -8910,7 +8910,7 @@
     </row>
     <row r="226">
       <c r="A226">
-        <v>1087</v>
+        <v>925</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     </row>
     <row r="227">
       <c r="A227">
-        <v>1088</v>
+        <v>926</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
@@ -8986,7 +8986,7 @@
     </row>
     <row r="228">
       <c r="A228">
-        <v>1089</v>
+        <v>927</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
@@ -9024,7 +9024,7 @@
     </row>
     <row r="229">
       <c r="A229">
-        <v>1091</v>
+        <v>929</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -9062,7 +9062,7 @@
     </row>
     <row r="230">
       <c r="A230">
-        <v>1092</v>
+        <v>930</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -9100,7 +9100,7 @@
     </row>
     <row r="231">
       <c r="A231">
-        <v>1093</v>
+        <v>931</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
     </row>
     <row r="232">
       <c r="A232">
-        <v>1094</v>
+        <v>932</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
@@ -9176,7 +9176,7 @@
     </row>
     <row r="233">
       <c r="A233">
-        <v>1095</v>
+        <v>933</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -9214,7 +9214,7 @@
     </row>
     <row r="234">
       <c r="A234">
-        <v>1097</v>
+        <v>935</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -9252,7 +9252,7 @@
     </row>
     <row r="235">
       <c r="A235">
-        <v>1098</v>
+        <v>936</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -9290,7 +9290,7 @@
     </row>
     <row r="236">
       <c r="A236">
-        <v>1099</v>
+        <v>937</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -9328,7 +9328,7 @@
     </row>
     <row r="237">
       <c r="A237">
-        <v>1100</v>
+        <v>938</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -9366,7 +9366,7 @@
     </row>
     <row r="238">
       <c r="A238">
-        <v>1101</v>
+        <v>939</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
@@ -9404,7 +9404,7 @@
     </row>
     <row r="239">
       <c r="A239">
-        <v>1102</v>
+        <v>940</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -9442,7 +9442,7 @@
     </row>
     <row r="240">
       <c r="A240">
-        <v>1103</v>
+        <v>941</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -9480,7 +9480,7 @@
     </row>
     <row r="241">
       <c r="A241">
-        <v>1104</v>
+        <v>942</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
@@ -9518,7 +9518,7 @@
     </row>
     <row r="242">
       <c r="A242">
-        <v>1105</v>
+        <v>943</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
@@ -9556,7 +9556,7 @@
     </row>
     <row r="243">
       <c r="A243">
-        <v>1107</v>
+        <v>945</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
     </row>
     <row r="244">
       <c r="A244">
-        <v>1108</v>
+        <v>946</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
@@ -9632,7 +9632,7 @@
     </row>
     <row r="245">
       <c r="A245">
-        <v>883</v>
+        <v>950</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -9670,7 +9670,7 @@
     </row>
     <row r="246">
       <c r="A246">
-        <v>666</v>
+        <v>956</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
@@ -9708,7 +9708,7 @@
     </row>
     <row r="247">
       <c r="A247">
-        <v>1024</v>
+        <v>970</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -9746,7 +9746,7 @@
     </row>
     <row r="248">
       <c r="A248">
-        <v>134</v>
+        <v>973</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -9784,7 +9784,7 @@
     </row>
     <row r="249">
       <c r="A249">
-        <v>962</v>
+        <v>974</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
@@ -9822,7 +9822,7 @@
     </row>
     <row r="250">
       <c r="A250">
-        <v>1196</v>
+        <v>977</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
@@ -9860,7 +9860,7 @@
     </row>
     <row r="251">
       <c r="A251">
-        <v>971</v>
+        <v>984</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
     </row>
     <row r="252">
       <c r="A252">
-        <v>972</v>
+        <v>985</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
     </row>
     <row r="253">
       <c r="A253">
-        <v>978</v>
+        <v>991</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
@@ -9974,7 +9974,7 @@
     </row>
     <row r="254">
       <c r="A254">
-        <v>143</v>
+        <v>1002</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
@@ -10012,7 +10012,7 @@
     </row>
     <row r="255">
       <c r="A255">
-        <v>502</v>
+        <v>1007</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -10050,7 +10050,7 @@
     </row>
     <row r="256">
       <c r="A256">
-        <v>1197</v>
+        <v>1009</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -10088,7 +10088,7 @@
     </row>
     <row r="257">
       <c r="A257">
-        <v>594</v>
+        <v>1010</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -10126,7 +10126,7 @@
     </row>
     <row r="258">
       <c r="A258">
-        <v>164</v>
+        <v>1014</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -10164,7 +10164,7 @@
     </row>
     <row r="259">
       <c r="A259">
-        <v>1409</v>
+        <v>1018</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -10202,7 +10202,7 @@
     </row>
     <row r="260">
       <c r="A260">
-        <v>1116</v>
+        <v>1019</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
@@ -10240,7 +10240,7 @@
     </row>
     <row r="261">
       <c r="A261">
-        <v>514</v>
+        <v>1022</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -10278,7 +10278,7 @@
     </row>
     <row r="262">
       <c r="A262">
-        <v>1393</v>
+        <v>1024</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -10316,7 +10316,7 @@
     </row>
     <row r="263">
       <c r="A263">
-        <v>1251</v>
+        <v>1026</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -10354,7 +10354,7 @@
     </row>
     <row r="264">
       <c r="A264">
-        <v>1263</v>
+        <v>1038</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -10392,7 +10392,7 @@
     </row>
     <row r="265">
       <c r="A265">
-        <v>1265</v>
+        <v>1040</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -10430,7 +10430,7 @@
     </row>
     <row r="266">
       <c r="A266">
-        <v>1283</v>
+        <v>1058</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -10468,7 +10468,7 @@
     </row>
     <row r="267">
       <c r="A267">
-        <v>1283</v>
+        <v>1058</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -10506,7 +10506,7 @@
     </row>
     <row r="268">
       <c r="A268">
-        <v>135</v>
+        <v>1059</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -10544,7 +10544,7 @@
     </row>
     <row r="269">
       <c r="A269">
-        <v>168</v>
+        <v>1062</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
     </row>
     <row r="270">
       <c r="A270">
-        <v>171</v>
+        <v>1065</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -10620,7 +10620,7 @@
     </row>
     <row r="271">
       <c r="A271">
-        <v>173</v>
+        <v>1067</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -10658,7 +10658,7 @@
     </row>
     <row r="272">
       <c r="A272">
-        <v>174</v>
+        <v>1068</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -10696,7 +10696,7 @@
     </row>
     <row r="273">
       <c r="A273">
-        <v>175</v>
+        <v>1069</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -10734,7 +10734,7 @@
     </row>
     <row r="274">
       <c r="A274">
-        <v>176</v>
+        <v>1070</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -10772,7 +10772,7 @@
     </row>
     <row r="275">
       <c r="A275">
-        <v>367</v>
+        <v>1071</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -10810,7 +10810,7 @@
     </row>
     <row r="276">
       <c r="A276">
-        <v>368</v>
+        <v>1072</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -10848,7 +10848,7 @@
     </row>
     <row r="277">
       <c r="A277">
-        <v>1227</v>
+        <v>1073</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -10886,7 +10886,7 @@
     </row>
     <row r="278">
       <c r="A278">
-        <v>1119</v>
+        <v>1080</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
@@ -10924,7 +10924,7 @@
     </row>
     <row r="279">
       <c r="A279">
-        <v>1125</v>
+        <v>1086</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -10962,7 +10962,7 @@
     </row>
     <row r="280">
       <c r="A280">
-        <v>1130</v>
+        <v>1091</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
@@ -11000,7 +11000,7 @@
     </row>
     <row r="281">
       <c r="A281">
-        <v>1132</v>
+        <v>1093</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
@@ -11038,7 +11038,7 @@
     </row>
     <row r="282">
       <c r="A282">
-        <v>505</v>
+        <v>1095</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
@@ -11076,7 +11076,7 @@
     </row>
     <row r="283">
       <c r="A283">
-        <v>506</v>
+        <v>1096</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
@@ -11114,7 +11114,7 @@
     </row>
     <row r="284">
       <c r="A284">
-        <v>1419</v>
+        <v>1099</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
@@ -11152,7 +11152,7 @@
     </row>
     <row r="285">
       <c r="A285">
-        <v>674</v>
+        <v>1106</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
@@ -11190,7 +11190,7 @@
     </row>
     <row r="286">
       <c r="A286">
-        <v>1014</v>
+        <v>1109</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
@@ -11228,7 +11228,7 @@
     </row>
     <row r="287">
       <c r="A287">
-        <v>596</v>
+        <v>1123</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
@@ -11266,7 +11266,7 @@
     </row>
     <row r="288">
       <c r="A288">
-        <v>369</v>
+        <v>1134</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
@@ -11304,7 +11304,7 @@
     </row>
     <row r="289">
       <c r="A289">
-        <v>1142</v>
+        <v>1135</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
@@ -11342,7 +11342,7 @@
     </row>
     <row r="290">
       <c r="A290">
-        <v>1143</v>
+        <v>1136</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
@@ -11380,7 +11380,7 @@
     </row>
     <row r="291">
       <c r="A291">
-        <v>1144</v>
+        <v>1137</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
@@ -11418,7 +11418,7 @@
     </row>
     <row r="292">
       <c r="A292">
-        <v>1146</v>
+        <v>1139</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
@@ -11456,7 +11456,7 @@
     </row>
     <row r="293">
       <c r="A293">
-        <v>1018</v>
+        <v>1162</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
@@ -11494,7 +11494,7 @@
     </row>
     <row r="294">
       <c r="A294">
-        <v>370</v>
+        <v>1166</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
@@ -11532,7 +11532,7 @@
     </row>
     <row r="295">
       <c r="A295">
-        <v>392</v>
+        <v>1168</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
@@ -11570,7 +11570,7 @@
     </row>
     <row r="296">
       <c r="A296">
-        <v>1287</v>
+        <v>1172</v>
       </c>
       <c r="B296" t="inlineStr">
         <is>
@@ -11608,7 +11608,7 @@
     </row>
     <row r="297">
       <c r="A297">
-        <v>1294</v>
+        <v>1178</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
@@ -11646,7 +11646,7 @@
     </row>
     <row r="298">
       <c r="A298">
-        <v>312</v>
+        <v>1196</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
@@ -11684,7 +11684,7 @@
     </row>
     <row r="299">
       <c r="A299">
-        <v>138</v>
+        <v>1198</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
@@ -11722,7 +11722,7 @@
     </row>
     <row r="300">
       <c r="A300">
-        <v>1308</v>
+        <v>1201</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
@@ -11760,7 +11760,7 @@
     </row>
     <row r="301">
       <c r="A301">
-        <v>1313</v>
+        <v>1206</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
@@ -11798,7 +11798,7 @@
     </row>
     <row r="302">
       <c r="A302">
-        <v>1315</v>
+        <v>1208</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
@@ -11836,7 +11836,7 @@
     </row>
     <row r="303">
       <c r="A303">
-        <v>1153</v>
+        <v>1209</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
@@ -11874,7 +11874,7 @@
     </row>
     <row r="304">
       <c r="A304">
-        <v>676</v>
+        <v>1225</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
@@ -11912,7 +11912,7 @@
     </row>
     <row r="305">
       <c r="A305">
-        <v>884</v>
+        <v>1229</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
@@ -11950,7 +11950,7 @@
     </row>
     <row r="306">
       <c r="A306">
-        <v>509</v>
+        <v>1230</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
@@ -11988,7 +11988,7 @@
     </row>
     <row r="307">
       <c r="A307">
-        <v>160</v>
+        <v>1240</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
@@ -12026,7 +12026,7 @@
     </row>
     <row r="308">
       <c r="A308">
-        <v>92</v>
+        <v>1242</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
@@ -12064,7 +12064,7 @@
     </row>
     <row r="309">
       <c r="A309">
-        <v>93</v>
+        <v>1243</v>
       </c>
       <c r="B309" t="inlineStr">
         <is>
@@ -12102,7 +12102,7 @@
     </row>
     <row r="310">
       <c r="A310">
-        <v>96</v>
+        <v>1246</v>
       </c>
       <c r="B310" t="inlineStr">
         <is>
@@ -12140,7 +12140,7 @@
     </row>
     <row r="311">
       <c r="A311">
-        <v>394</v>
+        <v>1248</v>
       </c>
       <c r="B311" t="inlineStr">
         <is>
@@ -12178,7 +12178,7 @@
     </row>
     <row r="312">
       <c r="A312">
-        <v>395</v>
+        <v>1249</v>
       </c>
       <c r="B312" t="inlineStr">
         <is>
@@ -12216,7 +12216,7 @@
     </row>
     <row r="313">
       <c r="A313">
-        <v>1229</v>
+        <v>1250</v>
       </c>
       <c r="B313" t="inlineStr">
         <is>
@@ -12254,7 +12254,7 @@
     </row>
     <row r="314">
       <c r="A314">
-        <v>270</v>
+        <v>1258</v>
       </c>
       <c r="B314" t="inlineStr">
         <is>
@@ -12292,7 +12292,7 @@
     </row>
     <row r="315">
       <c r="A315">
-        <v>273</v>
+        <v>1261</v>
       </c>
       <c r="B315" t="inlineStr">
         <is>
@@ -12330,7 +12330,7 @@
     </row>
     <row r="316">
       <c r="A316">
-        <v>276</v>
+        <v>1264</v>
       </c>
       <c r="B316" t="inlineStr">
         <is>
@@ -12368,7 +12368,7 @@
     </row>
     <row r="317">
       <c r="A317">
-        <v>359</v>
+        <v>1270</v>
       </c>
       <c r="B317" t="inlineStr">
         <is>
@@ -12406,7 +12406,7 @@
     </row>
     <row r="318">
       <c r="A318">
-        <v>1155</v>
+        <v>1277</v>
       </c>
       <c r="B318" t="inlineStr">
         <is>
@@ -12444,7 +12444,7 @@
     </row>
     <row r="319">
       <c r="A319">
-        <v>1156</v>
+        <v>1278</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
@@ -12482,7 +12482,7 @@
     </row>
     <row r="320">
       <c r="A320">
-        <v>184</v>
+        <v>1285</v>
       </c>
       <c r="B320" t="inlineStr">
         <is>
@@ -12520,7 +12520,7 @@
     </row>
     <row r="321">
       <c r="A321">
-        <v>185</v>
+        <v>1286</v>
       </c>
       <c r="B321" t="inlineStr">
         <is>
@@ -12558,7 +12558,7 @@
     </row>
     <row r="322">
       <c r="A322">
-        <v>776</v>
+        <v>1290</v>
       </c>
       <c r="B322" t="inlineStr">
         <is>
@@ -12596,7 +12596,7 @@
     </row>
     <row r="323">
       <c r="A323">
-        <v>784</v>
+        <v>1298</v>
       </c>
       <c r="B323" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="324">
       <c r="A324">
-        <v>684</v>
+        <v>1299</v>
       </c>
       <c r="B324" t="inlineStr">
         <is>
@@ -12672,7 +12672,7 @@
     </row>
     <row r="325">
       <c r="A325">
-        <v>840</v>
+        <v>1302</v>
       </c>
       <c r="B325" t="inlineStr">
         <is>
@@ -12710,7 +12710,7 @@
     </row>
     <row r="326">
       <c r="A326">
-        <v>1347</v>
+        <v>1320</v>
       </c>
       <c r="B326" t="inlineStr">
         <is>
@@ -12748,7 +12748,7 @@
     </row>
     <row r="327">
       <c r="A327">
-        <v>66</v>
+        <v>1358</v>
       </c>
       <c r="B327" t="inlineStr">
         <is>
@@ -12786,7 +12786,7 @@
     </row>
     <row r="328">
       <c r="A328">
-        <v>71</v>
+        <v>1363</v>
       </c>
       <c r="B328" t="inlineStr">
         <is>
@@ -12824,7 +12824,7 @@
     </row>
     <row r="329">
       <c r="A329">
-        <v>71</v>
+        <v>1363</v>
       </c>
       <c r="B329" t="inlineStr">
         <is>
@@ -12862,7 +12862,7 @@
     </row>
     <row r="330">
       <c r="A330">
-        <v>372</v>
+        <v>1368</v>
       </c>
       <c r="B330" t="inlineStr">
         <is>
@@ -12900,7 +12900,7 @@
     </row>
     <row r="331">
       <c r="A331">
-        <v>373</v>
+        <v>1369</v>
       </c>
       <c r="B331" t="inlineStr">
         <is>
@@ -12938,7 +12938,7 @@
     </row>
     <row r="332">
       <c r="A332">
-        <v>292</v>
+        <v>1371</v>
       </c>
       <c r="B332" t="inlineStr">
         <is>
@@ -12976,7 +12976,7 @@
     </row>
     <row r="333">
       <c r="A333">
-        <v>145</v>
+        <v>1375</v>
       </c>
       <c r="B333" t="inlineStr">
         <is>
@@ -13014,7 +13014,7 @@
     </row>
     <row r="334">
       <c r="A334">
-        <v>852</v>
+        <v>1378</v>
       </c>
       <c r="B334" t="inlineStr">
         <is>
@@ -13052,7 +13052,7 @@
     </row>
     <row r="335">
       <c r="A335">
-        <v>77</v>
+        <v>1408</v>
       </c>
       <c r="B335" t="inlineStr">
         <is>
@@ -13090,7 +13090,7 @@
     </row>
     <row r="336">
       <c r="A336">
-        <v>78</v>
+        <v>1409</v>
       </c>
       <c r="B336" t="inlineStr">
         <is>
@@ -13128,7 +13128,7 @@
     </row>
     <row r="337">
       <c r="A337">
-        <v>1425</v>
+        <v>1413</v>
       </c>
       <c r="B337" t="inlineStr">
         <is>
@@ -13166,7 +13166,7 @@
     </row>
     <row r="338">
       <c r="A338">
-        <v>1165</v>
+        <v>1415</v>
       </c>
       <c r="B338" t="inlineStr">
         <is>
@@ -13204,7 +13204,7 @@
     </row>
     <row r="339">
       <c r="A339">
-        <v>1165</v>
+        <v>1415</v>
       </c>
       <c r="B339" t="inlineStr">
         <is>
@@ -13242,7 +13242,7 @@
     </row>
     <row r="340">
       <c r="A340">
-        <v>1166</v>
+        <v>1416</v>
       </c>
       <c r="B340" t="inlineStr">
         <is>
@@ -13280,7 +13280,7 @@
     </row>
     <row r="341">
       <c r="A341">
-        <v>1166</v>
+        <v>1416</v>
       </c>
       <c r="B341" t="inlineStr">
         <is>

</xml_diff>